<commit_message>
original code bug fixes, file organization
</commit_message>
<xml_diff>
--- a/experiments/original/experiment_code/e1_stimuli.xlsx
+++ b/experiments/original/experiment_code/e1_stimuli.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bowdoin-my.sharepoint.com/personal/jsides_bowdoin_edu/Documents/Documents/lexicon_lab/object-state-changes/experiments/original/experiment_code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="200" documentId="13_ncr:1_{C493319E-5911-4547-B9FE-CD4AF22DD00F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5DDC72B-EBB1-464C-B148-22C9E7800551}"/>
+  <xr:revisionPtr revIDLastSave="234" documentId="13_ncr:1_{C493319E-5911-4547-B9FE-CD4AF22DD00F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32556ACA-AD67-2F42-8659-548C9D990747}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14280" windowHeight="18000" activeTab="3" xr2:uid="{5EADE905-632C-A04D-8302-0650934DE955}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{5EADE905-632C-A04D-8302-0650934DE955}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -1740,10 +1740,10 @@
         <v>172</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>258</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>176</v>
@@ -1752,10 +1752,10 @@
         <v>177</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -5617,10 +5617,10 @@
         <v>172</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>258</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>176</v>
@@ -5629,10 +5629,10 @@
         <v>177</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -9494,10 +9494,10 @@
         <v>172</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>258</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>176</v>
@@ -9506,10 +9506,10 @@
         <v>177</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -13372,10 +13372,10 @@
         <v>172</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>258</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>176</v>
@@ -13384,10 +13384,10 @@
         <v>177</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -18424,7 +18424,7 @@
         <v>255</v>
       </c>
       <c r="B98" s="3" t="str">
-        <f t="shared" ref="B98:B129" si="3">CONCATENATE("['",A98,"'],")</f>
+        <f t="shared" ref="B98:B101" si="3">CONCATENATE("['",A98,"'],")</f>
         <v>['PICTURES/watch.jpg'],</v>
       </c>
     </row>

</xml_diff>